<commit_message>
Extended data to 2070
</commit_message>
<xml_diff>
--- a/InputData/elec/DPbES/Dispatch Priority by Elec Source.xlsx
+++ b/InputData/elec/DPbES/Dispatch Priority by Elec Source.xlsx
@@ -1,21 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10526"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Meghan\Dropbox (Energy Innovation)\EPS Versions\eps-1.5.0-us-wipI\InputData\elec\DPbES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/elec/DPbES/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1F20E32-7502-3B46-AD7C-C66F2D49F394}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="90" windowWidth="22995" windowHeight="11055"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="DPbES" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -124,7 +138,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -189,9 +203,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -229,9 +243,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -266,7 +280,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -301,7 +315,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -474,86 +488,86 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>14</v>
       </c>
@@ -565,18 +579,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:AK17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:BE17"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.85546875" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="23.83203125" customWidth="1"/>
+    <col min="2" max="2" width="9.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:57" ht="32" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>32</v>
       </c>
@@ -688,8 +702,68 @@
       <c r="AK1">
         <v>2050</v>
       </c>
+      <c r="AL1">
+        <v>2051</v>
+      </c>
+      <c r="AM1">
+        <v>2052</v>
+      </c>
+      <c r="AN1">
+        <v>2053</v>
+      </c>
+      <c r="AO1">
+        <v>2054</v>
+      </c>
+      <c r="AP1">
+        <v>2055</v>
+      </c>
+      <c r="AQ1">
+        <v>2056</v>
+      </c>
+      <c r="AR1">
+        <v>2057</v>
+      </c>
+      <c r="AS1">
+        <v>2058</v>
+      </c>
+      <c r="AT1">
+        <v>2059</v>
+      </c>
+      <c r="AU1">
+        <v>2060</v>
+      </c>
+      <c r="AV1">
+        <v>2061</v>
+      </c>
+      <c r="AW1">
+        <v>2062</v>
+      </c>
+      <c r="AX1">
+        <v>2063</v>
+      </c>
+      <c r="AY1">
+        <v>2064</v>
+      </c>
+      <c r="AZ1">
+        <v>2065</v>
+      </c>
+      <c r="BA1">
+        <v>2066</v>
+      </c>
+      <c r="BB1">
+        <v>2067</v>
+      </c>
+      <c r="BC1">
+        <v>2068</v>
+      </c>
+      <c r="BD1">
+        <v>2069</v>
+      </c>
+      <c r="BE1">
+        <v>2070</v>
+      </c>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>26</v>
       </c>
@@ -836,8 +910,88 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
+      <c r="AL2">
+        <f>AK2</f>
+        <v>5</v>
+      </c>
+      <c r="AM2">
+        <f t="shared" ref="AM2:BE16" si="1">AL2</f>
+        <v>5</v>
+      </c>
+      <c r="AN2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AO2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AP2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AQ2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AR2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AS2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AT2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AU2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AV2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AW2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AX2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AY2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AZ2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="BA2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="BB2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="BC2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="BD2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="BE2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -845,67 +999,67 @@
         <v>4</v>
       </c>
       <c r="C3">
-        <f t="shared" ref="C3:R12" si="1">$B3</f>
+        <f t="shared" ref="C3:R12" si="2">$B3</f>
         <v>4</v>
       </c>
       <c r="D3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="E3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="F3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="G3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="H3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="I3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="J3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="K3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="L3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="M3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="N3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="O3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="P3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="Q3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="R3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="S3">
@@ -984,8 +1138,88 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
+      <c r="AL3">
+        <f t="shared" ref="AL3:BA17" si="3">AK3</f>
+        <v>4</v>
+      </c>
+      <c r="AM3">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="AN3">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="AO3">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="AP3">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="AQ3">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="AR3">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="AS3">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="AT3">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="AU3">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="AV3">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="AW3">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="AX3">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="AY3">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="AZ3">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="BA3">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="BB3">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="BC3">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="BD3">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="BE3">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -993,7 +1227,7 @@
         <v>3</v>
       </c>
       <c r="C4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="D4">
@@ -1132,8 +1366,88 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
+      <c r="AL4">
+        <f t="shared" si="3"/>
+        <v>3</v>
+      </c>
+      <c r="AM4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AN4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AO4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AP4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AQ4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AR4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AS4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AT4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AU4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AV4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AW4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AX4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AY4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AZ4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="BA4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="BB4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="BC4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="BD4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="BE4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1141,7 +1455,7 @@
         <v>2</v>
       </c>
       <c r="C5">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="D5">
@@ -1280,8 +1594,88 @@
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
+      <c r="AL5">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="AM5">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AN5">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AO5">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AP5">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AQ5">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AR5">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AS5">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AT5">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AU5">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AV5">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AW5">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AX5">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AY5">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AZ5">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BA5">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BB5">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BC5">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BD5">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BE5">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -1289,7 +1683,7 @@
         <v>2</v>
       </c>
       <c r="C6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="D6">
@@ -1428,8 +1822,88 @@
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
+      <c r="AL6">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="AM6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AN6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AO6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AP6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AQ6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AR6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AS6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AT6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AU6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AV6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AW6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AX6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AY6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AZ6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BA6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BB6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BC6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BD6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BE6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1437,7 +1911,7 @@
         <v>2</v>
       </c>
       <c r="C7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="D7">
@@ -1576,8 +2050,88 @@
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
+      <c r="AL7">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="AM7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AN7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AO7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AP7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AQ7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AR7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AS7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AT7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AU7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AV7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AW7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AX7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AY7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AZ7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BA7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BB7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BC7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BD7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BE7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
     </row>
-    <row r="8" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -1585,7 +2139,7 @@
         <v>2</v>
       </c>
       <c r="C8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="D8">
@@ -1724,8 +2278,88 @@
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
+      <c r="AL8">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="AM8">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AN8">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AO8">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AP8">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AQ8">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AR8">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AS8">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AT8">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AU8">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AV8">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AW8">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AX8">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AY8">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AZ8">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BA8">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BB8">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BC8">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BD8">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BE8">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
     </row>
-    <row r="9" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -1733,7 +2367,7 @@
         <v>3</v>
       </c>
       <c r="C9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="D9">
@@ -1865,15 +2499,95 @@
         <v>3</v>
       </c>
       <c r="AJ9">
-        <f t="shared" ref="D9:AK12" si="2">$B9</f>
+        <f t="shared" ref="D9:AK12" si="4">$B9</f>
         <v>3</v>
       </c>
       <c r="AK9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
+        <v>3</v>
+      </c>
+      <c r="AL9">
+        <f t="shared" si="3"/>
+        <v>3</v>
+      </c>
+      <c r="AM9">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AN9">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AO9">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AP9">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AQ9">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AR9">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AS9">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AT9">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AU9">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AV9">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AW9">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AX9">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AY9">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="AZ9">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="BA9">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="BB9">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="BC9">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="BD9">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="BE9">
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -1881,147 +2595,227 @@
         <v>2</v>
       </c>
       <c r="C10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="D10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="E10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="F10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="G10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="H10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="I10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="J10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="K10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="L10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="M10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="N10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="O10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="P10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="Q10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="R10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="S10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="T10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="U10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="V10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="W10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="X10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="Y10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="Z10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="AA10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="AB10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="AC10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="AD10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="AE10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="AF10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="AG10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="AH10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="AI10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="AJ10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="AK10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+      <c r="AL10">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="AM10">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AN10">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AO10">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AP10">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AQ10">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AR10">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AS10">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AT10">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AU10">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AV10">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AW10">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AX10">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AY10">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AZ10">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BA10">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BB10">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BC10">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BD10">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BE10">
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -2029,147 +2823,227 @@
         <v>1</v>
       </c>
       <c r="C11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="D11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="E11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="F11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="G11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="H11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="J11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="K11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="L11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="M11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="N11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="O11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="P11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="Q11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="R11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="S11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="T11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="U11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="V11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="W11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="X11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="Y11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="Z11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AA11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AB11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AC11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AD11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AE11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AF11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AG11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AH11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AI11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AJ11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AK11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AL11">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="AM11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AN11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AO11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AP11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AQ11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AR11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AS11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AT11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AU11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AV11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AW11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AX11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AY11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AZ11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="BA11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="BB11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="BC11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="BD11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="BE11">
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -2177,147 +3051,227 @@
         <v>1</v>
       </c>
       <c r="C12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="D12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="E12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="F12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="G12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="H12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="J12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="K12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="L12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="M12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="N12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="O12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="P12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="Q12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="R12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="S12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="T12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="U12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="V12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="W12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="X12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="Y12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="Z12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AA12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AB12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AC12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AD12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AE12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AF12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AG12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AH12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AI12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AJ12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AK12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AL12">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="AM12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AN12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AO12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AP12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AQ12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AR12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AS12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AT12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AU12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AV12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AW12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AX12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AY12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AZ12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="BA12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="BB12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="BC12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="BD12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="BE12">
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -2326,147 +3280,227 @@
         <v>5</v>
       </c>
       <c r="C13">
-        <f t="shared" ref="C13:AK13" si="3">C2</f>
+        <f t="shared" ref="C13:AK13" si="5">C2</f>
         <v>5</v>
       </c>
       <c r="D13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="K13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="L13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="M13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="N13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="O13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="P13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="Q13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="R13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="S13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="T13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="U13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="V13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="W13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="X13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="Y13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="Z13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="AA13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="AB13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="AC13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="AD13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="AE13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="AF13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="AG13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="AH13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="AI13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="AJ13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="AK13">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="AL13">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="E13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="F13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="G13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="H13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="I13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="J13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="K13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="L13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="M13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="N13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="O13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="P13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="Q13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="R13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="S13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="T13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="U13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="V13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="W13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="X13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="Y13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="Z13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="AA13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="AB13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="AC13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="AD13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="AE13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="AF13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="AG13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="AH13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="AI13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="AJ13">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="AK13">
-        <f t="shared" si="3"/>
+      <c r="AM13">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AN13">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AO13">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AP13">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AQ13">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AR13">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AS13">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AT13">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AU13">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AV13">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AW13">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AX13">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AY13">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="AZ13">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="BA13">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="BB13">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="BC13">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="BD13">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="BE13">
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>28</v>
       </c>
@@ -2475,147 +3509,227 @@
         <v>2</v>
       </c>
       <c r="C14">
-        <f t="shared" ref="C14:AK14" si="4">C6</f>
+        <f t="shared" ref="C14:AK14" si="6">C6</f>
         <v>2</v>
       </c>
       <c r="D14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="E14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="F14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="G14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="H14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="I14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="J14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="K14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="L14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="M14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="N14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="O14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="P14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="Q14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="R14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="S14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="T14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="U14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="V14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="W14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="X14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="Y14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="Z14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="AA14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="AB14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="AC14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="AD14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="AE14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="AF14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="AG14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="AH14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="AI14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="AJ14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="AK14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
+        <v>2</v>
+      </c>
+      <c r="AL14">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="AM14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AN14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AO14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AP14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AQ14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AR14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AS14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AT14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AU14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AV14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AW14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AX14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AY14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="AZ14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BA14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BB14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BC14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BD14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="BE14">
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>29</v>
       </c>
@@ -2624,147 +3738,227 @@
         <v>1</v>
       </c>
       <c r="C15">
-        <f t="shared" ref="C15:AK15" si="5">C11</f>
+        <f t="shared" ref="C15:AK15" si="7">C11</f>
         <v>1</v>
       </c>
       <c r="D15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="E15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="F15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="G15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="H15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="I15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="J15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="K15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="L15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="M15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="N15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="O15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="P15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="Q15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="R15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="S15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="T15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="U15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="V15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="W15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="X15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="Y15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="Z15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AA15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AB15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AC15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AD15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AE15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AF15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AG15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AH15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AI15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AJ15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AK15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="AL15">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="AM15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AN15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AO15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AP15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AQ15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AR15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AS15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AT15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AU15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AV15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AW15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AX15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AY15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AZ15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="BA15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="BB15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="BC15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="BD15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="BE15">
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -2773,147 +3967,227 @@
         <v>1</v>
       </c>
       <c r="C16">
-        <f t="shared" ref="C16:AK16" si="6">C11</f>
+        <f t="shared" ref="C16:AK16" si="8">C11</f>
         <v>1</v>
       </c>
       <c r="D16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="E16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="F16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="G16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="H16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="I16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="J16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="K16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="L16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="M16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="N16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="O16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="P16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="Q16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="R16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="S16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="T16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="U16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="V16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="W16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="X16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="Y16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="Z16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AA16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AB16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AC16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AD16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AE16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AF16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AG16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AH16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AI16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AJ16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AK16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="AL16">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="AM16">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AN16">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AO16">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AP16">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AQ16">
+        <f t="shared" ref="AM16:BE17" si="9">AP16</f>
+        <v>1</v>
+      </c>
+      <c r="AR16">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="AS16">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="AT16">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="AU16">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="AV16">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="AW16">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="AX16">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="AY16">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="AZ16">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="BA16">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="BB16">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="BC16">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="BD16">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="BE16">
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>31</v>
       </c>
@@ -2922,143 +4196,223 @@
         <v>3</v>
       </c>
       <c r="C17">
-        <f t="shared" ref="C17:AK17" si="7">C9</f>
+        <f t="shared" ref="C17:AK17" si="10">C9</f>
         <v>3</v>
       </c>
       <c r="D17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="E17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="F17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="G17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="H17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="I17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="J17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="K17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="L17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="M17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="N17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="O17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="P17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="Q17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="R17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="S17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="T17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="U17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="V17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="W17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="X17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="Y17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="Z17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="AA17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="AB17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="AC17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="AD17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="AE17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="AF17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="AG17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="AH17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="AI17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="AJ17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
       <c r="AK17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
+        <v>3</v>
+      </c>
+      <c r="AL17">
+        <f t="shared" si="3"/>
+        <v>3</v>
+      </c>
+      <c r="AM17">
+        <f t="shared" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="AN17">
+        <f t="shared" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="AO17">
+        <f t="shared" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="AP17">
+        <f t="shared" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="AQ17">
+        <f t="shared" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="AR17">
+        <f t="shared" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="AS17">
+        <f t="shared" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="AT17">
+        <f t="shared" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="AU17">
+        <f t="shared" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="AV17">
+        <f t="shared" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="AW17">
+        <f t="shared" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="AX17">
+        <f t="shared" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="AY17">
+        <f t="shared" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="AZ17">
+        <f t="shared" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="BA17">
+        <f t="shared" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="BB17">
+        <f t="shared" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="BC17">
+        <f t="shared" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="BD17">
+        <f t="shared" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="BE17">
+        <f t="shared" si="9"/>
         <v>3</v>
       </c>
     </row>

</xml_diff>